<commit_message>
Vuelvo a ignorar los .pkl
</commit_message>
<xml_diff>
--- a/data/italy/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/italy/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,45 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>z3jsi9f5</t>
+          <t>x8OGzlAO</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45569.5625</v>
+        <v>45571.3125</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">feliciani e 
+          <t xml:space="preserve">marinelli l 
   ita </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio diego armando maradona
-  naples </t>
+          <t xml:space="preserve">allianz stadium
+  turin </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>54726</v>
+        <v>41507</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>69Dxbc61</t>
+          <t>C06aJvIB</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ttyLthOA</t>
+          <t>SCGVmKHb</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,45 +574,45 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>8SWavWAa</t>
+          <t>dzYLoEIP</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45569.65625</v>
+        <v>45571.41666666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">guida m 
+          <t xml:space="preserve">di bello m 
   ita </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio marc antonio bentegodi
-  verona </t>
+          <t xml:space="preserve">stadio renato dall ara
+  bologna </t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>39211</v>
+        <v>38279</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>rJVAIaHo</t>
+          <t>0M9xNN8N</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>MkPmVv50</t>
+          <t>6DxlaxHN</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -641,45 +641,45 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>WUqjkmPH</t>
+          <t>SW3Qfiet</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45570.41666666666</v>
+        <v>45571.41666666666</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">mariani m 
+          <t xml:space="preserve">ayroldi g 
   ita </t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">bluenergy stadium   stadio friuli
-  udine </t>
+          <t xml:space="preserve">stadio olimpico
+  rome </t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>25144</v>
+        <v>70634</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>rXw8YKDE</t>
+          <t>URcSl02h</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>G8lYsMgU</t>
+          <t>0ESCnI1H</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -708,45 +708,45 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>EB8yv2aJ</t>
+          <t>lnhZhVPh</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45570.54166666666</v>
+        <v>45571.54166666666</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">chiffi d 
+          <t xml:space="preserve">la penna f 
   ita </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">gewiss stadium
-  bergamo </t>
+          <t xml:space="preserve">brianteo
+  monza </t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>24950</v>
+        <v>17102</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>8C9JjMXu</t>
+          <t>4YSMlwj7</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>d0PJxeie</t>
+          <t>zVqqL0ma</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -775,45 +775,45 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>ttV7xAuC</t>
+          <t>SIOithtm</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45570.65625</v>
+        <v>45571.65625</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">marcenaro m 
+          <t xml:space="preserve">pairetto l 
   ita </t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio giuseppe meazza  san siro 
-  milan </t>
+          <t xml:space="preserve">stadio artemio franchi
+  florence </t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>80018</v>
+        <v>43147</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Iw7eKK25</t>
+          <t>Q3A3IbXH</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>MZFZnvX4</t>
+          <t>8Sa8HInO</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -842,45 +842,40 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>x8OGzlAO</t>
+          <t>Cl5M5C3L</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45571.3125</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">marinelli l 
-  ita </t>
-        </is>
-      </c>
+        <v>45584.41666666666</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">allianz stadium
-  turin </t>
+          <t xml:space="preserve">stadio giuseppe sinigaglia
+  como </t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>41507</v>
+        <v>13602</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>C06aJvIB</t>
+          <t>ttyLthOA</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>como</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SCGVmKHb</t>
+          <t>6DxlaxHN</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -909,45 +904,40 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>dzYLoEIP</t>
+          <t>EXLhbUee</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45571.41666666666</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">di bello m 
-  ita </t>
-        </is>
-      </c>
+        <v>45584.41666666666</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio renato dall ara
-  bologna </t>
+          <t xml:space="preserve">stadio luigi ferraris
+  genoa </t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>38279</v>
+        <v>36599</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>d0PJxeie</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>genoa</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>0M9xNN8N</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>bologna</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>6DxlaxHN</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>parma</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -976,45 +966,40 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>SW3Qfiet</t>
+          <t>SznSCTAl</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45571.41666666666</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ayroldi g 
-  ita </t>
-        </is>
-      </c>
+        <v>45584.54166666666</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio olimpico
-  rome </t>
+          <t xml:space="preserve">stadio giuseppe meazza  san siro 
+  milan </t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>70634</v>
+        <v>80018</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>URcSl02h</t>
+          <t>8Sa8HInO</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0ESCnI1H</t>
+          <t>rXw8YKDE</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -1043,45 +1028,40 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>lnhZhVPh</t>
+          <t>2g2mKBIE</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45571.54166666666</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">la penna f 
-  ita </t>
-        </is>
-      </c>
+        <v>45584.65625</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">brianteo
-  monza </t>
+          <t xml:space="preserve">allianz stadium
+  turin </t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>17102</v>
+        <v>41507</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4YSMlwj7</t>
+          <t>C06aJvIB</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>zVqqL0ma</t>
+          <t>URcSl02h</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1110,45 +1090,40 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>SIOithtm</t>
+          <t>8Kjh0jRr</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45571.65625</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pairetto l 
-  ita </t>
-        </is>
-      </c>
+        <v>45585.3125</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio artemio franchi
-  florence </t>
+          <t xml:space="preserve">stadio carlo castellani
+  empoli </t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>43147</v>
+        <v>16284</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Q3A3IbXH</t>
+          <t>0ESCnI1H</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>8Sa8HInO</t>
+          <t>69Dxbc61</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1177,40 +1152,40 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Cl5M5C3L</t>
+          <t>AJ5eIkmR</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45584.41666666666</v>
+        <v>45585.41666666666</v>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio giuseppe sinigaglia
-  como </t>
+          <t xml:space="preserve">stadio via del mare
+  lecce </t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>13602</v>
+        <v>40670</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ttyLthOA</t>
+          <t>G8lYsMgU</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>6DxlaxHN</t>
+          <t>Q3A3IbXH</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1239,40 +1214,40 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>EXLhbUee</t>
+          <t>dGwq9oAD</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45584.41666666666</v>
+        <v>45585.41666666666</v>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">stadio luigi ferraris
-  genoa </t>
+          <t xml:space="preserve">stadio pierluigi penzo
+  venice </t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>36599</v>
+        <v>11150</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>d0PJxeie</t>
+          <t>MkPmVv50</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0M9xNN8N</t>
+          <t>8C9JjMXu</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1293,6 +1268,130 @@
         </is>
       </c>
       <c r="O13" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>GMBD7YY8</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45585.54166666666</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unipol domus
+  cagliari </t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>16416</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SCGVmKHb</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>cagliari</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>MZFZnvX4</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>torino</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>77</v>
+      </c>
+      <c r="K14" t="n">
+        <v>771</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>0lpzB7u1</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45585.65625</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stadio olimpico
+  rome </t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>70634</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>zVqqL0ma</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>as roma</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Iw7eKK25</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>inter</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>77</v>
+      </c>
+      <c r="K15" t="n">
+        <v>771</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
         <is>
           <t>serie a</t>
         </is>

</xml_diff>